<commit_message>
auto: 작업 자동 저장 2026-08-06 11:56
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/EE/05_unified_ledger/EE_골든셋_통합대장_13문항_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/EE/05_unified_ledger/EE_골든셋_통합대장_13문항_v1_0.xlsx
@@ -1272,7 +1272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1295,7 +1295,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>재료 풀</t>
+          <t>재료 풀(대표 추출)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1312,7 +1312,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>직접 커버(전 차수)</t>
+          <t>직접 커버(풀 내)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1329,7 +1329,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>흡수</t>
+          <t>선외 추가 커버</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1339,14 +1339,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>명단 갱신 이전 차수 확보분 — 소실 아님(추가 확보)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>부적격</t>
+          <t>흡수</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1356,14 +1356,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미출제 단위</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>잔여</t>
+          <t>부적격</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1373,22 +1373,39 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>마감</t>
+          <t>미출제 단위</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>등식: 12+0+0+0=12</t>
+          <t>잔여</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>마감</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>등식: 12+0+0+0=12 (+선외 0)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>소실 0(assert)</t>
         </is>

</xml_diff>